<commit_message>
Add all untracked files - data, reports, coverage, cache, migrations
- Add new data files: All_Projects.XLSX, CJI3 formatted reports, project analysis outputs
- Add coverage reports (htmlcov), pytest cache, and backups
- Add Claude settings, PROJECT_ANALYSIS_UPDATE.md, VISUALIZATION_GUIDE.md
- Add uploaded data files and staticfiles
- Add compiled pycache files across all modules

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Code/data/reports/CrossTab_Report.xlsx
+++ b/Code/data/reports/CrossTab_Report.xlsx
@@ -182,9 +182,7 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -703,34 +701,30 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>NIGEL</t>
+          <t>NIRL</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>NIRL</t>
+          <t>NLCIL</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>NLCIL</t>
+          <t>NTPL</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
-          <t>NTPL</t>
+          <t>NUPPL</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>NUPPL</t>
-        </is>
-      </c>
-      <c r="G1" s="8" t="inlineStr">
-        <is>
           <t>Total</t>
         </is>
       </c>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -739,23 +733,21 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E2" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" s="15" t="n">
-        <v>46</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="G2" s="15" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -767,20 +759,18 @@
         <v>0</v>
       </c>
       <c r="C3" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="12" t="n">
-        <v>6</v>
-      </c>
       <c r="E3" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="15" t="n">
         <v>7</v>
       </c>
+      <c r="G3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -792,20 +782,18 @@
         <v>0</v>
       </c>
       <c r="C4" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>1</v>
-      </c>
       <c r="F4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="15" t="n">
         <v>11</v>
       </c>
+      <c r="G4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -817,20 +805,18 @@
         <v>0</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="15" t="n">
         <v>56</v>
       </c>
+      <c r="G5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -842,20 +828,18 @@
         <v>0</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="15" t="n">
         <v>2</v>
       </c>
+      <c r="G6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -867,20 +851,18 @@
         <v>0</v>
       </c>
       <c r="C7" s="11" t="n">
+        <v>305</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="12" t="n">
-        <v>305</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>1</v>
-      </c>
       <c r="F7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="15" t="n">
         <v>306</v>
       </c>
+      <c r="G7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -889,23 +871,21 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C8" s="11" t="n">
+        <v>405</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="12" t="n">
-        <v>405</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <v>10</v>
-      </c>
       <c r="F8" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="15" t="n">
-        <v>428</v>
-      </c>
+        <v>427</v>
+      </c>
+      <c r="G8" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">

</xml_diff>